<commit_message>
Add official structural sources and data catalog
</commit_message>
<xml_diff>
--- a/metadata/data_gap_analysis.xlsx
+++ b/metadata/data_gap_analysis.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Gap Analysis" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Gap Analysis'!$A$1:$N$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Gap Analysis'!$A$1:$N$29</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -32,7 +32,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -51,22 +51,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00D9EAF7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F4CCCC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E4DFEC"/>
       </patternFill>
     </fill>
     <fill>
@@ -87,7 +77,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -103,12 +93,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -476,18 +460,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N44"/>
+  <dimension ref="A1:N29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="23" customWidth="1" min="3" max="3"/>
-    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
     <col width="23" customWidth="1" min="5" max="5"/>
     <col width="37" customWidth="1" min="6" max="6"/>
     <col width="42" customWidth="1" min="7" max="7"/>
     <col width="42" customWidth="1" min="8" max="8"/>
-    <col width="42" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
     <col width="42" customWidth="1" min="10" max="10"/>
     <col width="22" customWidth="1" min="11" max="11"/>
     <col width="20" customWidth="1" min="12" max="12"/>
@@ -630,12 +614,12 @@
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>Provider model series; values and history may be revised.</t>
+          <t>Provider modeled index; histories can be revised.</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>Keep as the primary monthly local home-value series.</t>
+          <t>Keep as the local home-value index.</t>
         </is>
       </c>
     </row>
@@ -657,7 +641,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Federal Housing Finance Agency</t>
+          <t>FHFA</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -672,7 +656,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>analytics.state_quarterly_panel|analytics.metro_quarterly_panel|analytics.county_annual_structural</t>
+          <t>analytics.state_quarterly_panel|analytics.metro_quarterly_panel|analytics.county_annual_controls</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -707,7 +691,7 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>Retain at native frequency and rebuild through the pipeline.</t>
+          <t>Retain at native frequency.</t>
         </is>
       </c>
     </row>
@@ -774,12 +758,12 @@
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>Transaction mix can change the median; historical values may be revised.</t>
+          <t>Transaction mix can change the median.</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>Retain the existing county series.</t>
+          <t>Retain as a transaction-price indicator.</t>
         </is>
       </c>
     </row>
@@ -846,12 +830,12 @@
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>County inventory is distinct from the ZIP Key Metrics active-listings field.</t>
+          <t>For-sale inventory only; not rental inventory.</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>Retain the existing county field and terminology.</t>
+          <t>Keep the label explicit.</t>
         </is>
       </c>
     </row>
@@ -881,9 +865,9 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>Partially implemented</t>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -918,12 +902,12 @@
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>Available at ZIP level as overlapping rolling-three-month observations; not interchangeable with county inventory.</t>
+          <t>ZIP product uses overlapping rolling-three-month windows.</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>Keep the separate ZIP field and do not relabel it as inventory.</t>
+          <t>Keep separate from county inventory.</t>
         </is>
       </c>
     </row>
@@ -990,12 +974,12 @@
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>Provider ratio; not additive and subject to revision.</t>
+          <t>Provider ratio; not additive.</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>Retain the existing county series.</t>
+          <t>Retain provider value.</t>
         </is>
       </c>
     </row>
@@ -1032,7 +1016,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>analytics.county_monthly_panel</t>
+          <t>analytics.county_monthly_panel|analytics.zip_monthly_panel</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -1042,12 +1026,12 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>monthly</t>
+          <t>monthly and rolling 3 months</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Los Angeles County</t>
+          <t>Los Angeles County and postal ZIPs</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1062,12 +1046,12 @@
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>Flow measure; ZIP product uses overlapping rolling-three-month windows.</t>
+          <t>ZIP observations are rolling windows.</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>Retain county monthly and separately labeled ZIP rolling series.</t>
+          <t>Use county monthly for time-series models.</t>
         </is>
       </c>
     </row>
@@ -1104,7 +1088,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>analytics.county_monthly_panel</t>
+          <t>analytics.county_monthly_panel|analytics.zip_monthly_panel</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -1114,12 +1098,12 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>monthly</t>
+          <t>monthly and rolling 3 months</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Los Angeles County</t>
+          <t>Los Angeles County and postal ZIPs</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1134,29 +1118,29 @@
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>Closed-sales flow; ZIP product uses overlapping rolling-three-month windows.</t>
+          <t>Closed-sales flow; ZIP observations are rolling windows.</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>Retain county monthly and separately labeled ZIP rolling series.</t>
+          <t>Use with inventory ratios.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>pending sales</t>
+          <t>days on market</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Homeowner</t>
+          <t>Overall housing market</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Leading indicator</t>
+          <t>Market time</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -1176,22 +1160,22 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>analytics.county_monthly_panel</t>
+          <t>analytics.county_monthly_panel|analytics.zip_monthly_panel</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>pending_sales</t>
+          <t>days_on_market|median_days_on_market</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>monthly</t>
+          <t>monthly and rolling 3 months</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Los Angeles County</t>
+          <t>Los Angeles County and postal ZIPs</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1206,29 +1190,29 @@
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>Provider series may be revised; ZIP observations are rolling windows.</t>
+          <t>Median; not additive.</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>Retain the existing series.</t>
+          <t>Expose as market-time indicator.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>days on market</t>
+          <t>share with price drops</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Homeowner</t>
+          <t>Overall housing market</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Market time</t>
+          <t>Leading indicator</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -1253,7 +1237,7 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>days_on_market</t>
+          <t>price_drop_share</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
@@ -1278,19 +1262,19 @@
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>Provider median and not additive.</t>
+          <t>Share, not count.</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>Retain the existing series.</t>
+          <t>Retain nulls and document coverage.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>share with price drops</t>
+          <t>30-year mortgage rate</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1300,12 +1284,12 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Leading indicator</t>
+          <t>Control</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Redfin Data Center</t>
+          <t>Freddie Mac PMMS</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -1325,44 +1309,44 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>price_drop_share</t>
+          <t>mortgage_rate_30y_monthly_average</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>monthly</t>
+          <t>weekly aggregated to monthly</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Los Angeles County</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>2012-01-31</t>
+          <t>1971-04-02</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>One source month is null; metric is a share and not a count.</t>
+          <t>National rate; not local.</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>Retain null and document coverage.</t>
+          <t>Keep U.S. geography explicit.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>30-year mortgage rate</t>
+          <t>single-family permits</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -1372,12 +1356,12 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>Supply</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Freddie Mac PMMS</t>
+          <t>Census BPS</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -1397,44 +1381,44 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>mortgage_rate_30y_monthly_average</t>
+          <t>permits_1_unit</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>weekly aggregated to monthly</t>
+          <t>monthly</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Los Angeles County</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>1971-04-02</t>
+          <t>2000-01-31</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>National rate is a control and must not be labeled as a Los Angeles rate.</t>
+          <t>Permits are authorizations, not starts or completions.</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>Retain weekly observations and explicit monthly mean/month-end constructions.</t>
+          <t>Retain as the single-family supply proxy.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>single-family permits</t>
+          <t>monthly mortgage payment</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1444,12 +1428,12 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Supply</t>
+          <t>Constructed indicator</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>U.S. Census Building Permits Survey</t>
+          <t>Redfin and Freddie Mac</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -1457,9 +1441,9 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>Implemented</t>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>Constructed variable</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -1469,7 +1453,7 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>permits_1_unit</t>
+          <t>mortgage_payment_10pct_down|mortgage_payment_20pct_down</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -1479,12 +1463,12 @@
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Los Angeles County</t>
+          <t>Los Angeles County with U.S. rate</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>2000-01-31</t>
+          <t>2012-01-31</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
@@ -1494,34 +1478,34 @@
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>Permits are authorizations, not starts or completions; methodology changed in 2022.</t>
+          <t>Principal-and-interest scenarios exclude taxes, insurance, HOA, maintenance, and mortgage insurance.</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>Retain reported/imputed flags and archive vintages.</t>
+          <t>Keep scenario assumptions visible.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>monthly mortgage payment</t>
+          <t>ZORI</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Homeowner</t>
+          <t>Renter</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Constructed indicator</t>
+          <t>Outcome</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Redfin median sale price and Freddie Mac PMMS</t>
+          <t>Zillow Research</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1529,9 +1513,9 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F15" s="5" t="inlineStr">
-        <is>
-          <t>Constructed variable</t>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -1541,7 +1525,7 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>mortgage_payment_10pct_down|mortgage_payment_20pct_down</t>
+          <t>zori</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
@@ -1551,12 +1535,12 @@
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>Los Angeles County with U.S. rate</t>
+          <t>Los Angeles County</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>2012-01-31</t>
+          <t>2015-01-31</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
@@ -1566,24 +1550,24 @@
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>Principal-and-interest scenarios exclude taxes, insurance, HOA, maintenance, and mortgage insurance.</t>
+          <t>Smoothed seasonally adjusted rent index; not inventory.</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>Retain explicit assumptions and scenario names.</t>
+          <t>Use as primary rent index.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>mortgage payment-to-rent</t>
+          <t>rent growth</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Homeowner</t>
+          <t>Renter</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1593,7 +1577,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Redfin, Freddie Mac, and Zillow</t>
+          <t>Zillow ZORI</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1601,7 +1585,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F16" s="5" t="inlineStr">
+      <c r="F16" s="4" t="inlineStr">
         <is>
           <t>Constructed variable</t>
         </is>
@@ -1613,7 +1597,7 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>mortgage_payment_to_rent_10pct_down|mortgage_payment_to_rent_20pct_down</t>
+          <t>zori_growth_mom|zori_growth_yoy</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -1628,7 +1612,7 @@
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>2015-01-31</t>
+          <t>2015-02-28</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
@@ -1638,106 +1622,90 @@
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>Combines transaction-price payment scenarios with an observed-rent index.</t>
+          <t>Depends on the active SA ZORI vintage.</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>Retain explicit construction and component vintages.</t>
+          <t>Rebuild when ZORI refreshes.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>price-to-income</t>
+          <t>rental inventory</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Homeowner</t>
+          <t>Renter</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Affordability</t>
+          <t>Supply</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>ACS and/or BEA</t>
+          <t>No verified official public source</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>Constructed variable</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>analytics.county_annual_structural|analytics.zcta_annual_structural</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t>annual_price_to_income_ratio</t>
-        </is>
-      </c>
+          <t>Missing — no verified public source</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr"/>
+      <c r="H17" s="2" t="inlineStr"/>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>annual</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>Los Angeles County</t>
-        </is>
-      </c>
-      <c r="K17" s="2" t="inlineStr">
-        <is>
-          <t>2024-12-31</t>
-        </is>
-      </c>
-      <c r="L17" s="2" t="inlineStr">
-        <is>
-          <t>2024-12-31</t>
-        </is>
-      </c>
+          <t>Los Angeles County or ZIPs</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr"/>
+      <c r="L17" s="2" t="inlineStr"/>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>A valid denominator is annual; monthly interpolation would create artificial precision.</t>
+          <t>ZORI measures rent levels and cannot serve as rental inventory.</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>Retain at native frequency and rebuild through the pipeline.</t>
+          <t>Leave unavailable until a documented public source is verified.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>housing turnover</t>
+          <t>rental vacancy</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Homeowner</t>
+          <t>Renter</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Constructed indicator</t>
+          <t>Supply</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Redfin homes sold and ACS housing stock</t>
+          <t>Census HVS</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1745,56 +1713,56 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F18" s="5" t="inlineStr">
-        <is>
-          <t>Constructed variable</t>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>analytics.county_annual_structural</t>
+          <t>analytics.state_quarterly_panel|analytics.metro_quarterly_panel</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>sales_to_housing_stock_turnover</t>
+          <t>hvs_rental_vacancy_rate_ca|hvs_rental_vacancy_rate_la_metro</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>monthly numerator and annual denominator</t>
+          <t>quarterly</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>Los Angeles County</t>
+          <t>California and published metro geographies</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>2024-12-31</t>
+          <t>2005-03-31</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>2024-12-31</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>Sales are present but a housing-stock denominator is not yet loaded.</t>
+          <t>Los Angeles County is not an HVS published geography; sampling uncertainty is retained.</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>Retain at native frequency and rebuild through the pipeline.</t>
+          <t>Retain native geography/frequency.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>ZORI</t>
+          <t>multifamily permits</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1804,12 +1772,12 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Outcome</t>
+          <t>Supply</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Zillow Research</t>
+          <t>Census BPS</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -1829,7 +1797,7 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>zori</t>
+          <t>permits_5_plus_units</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
@@ -1844,7 +1812,7 @@
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>2015-01-31</t>
+          <t>2000-01-31</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
@@ -1854,24 +1822,24 @@
       </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>Smoothed seasonally adjusted rent index; it is not rental inventory.</t>
+          <t>Permits are authorizations, not completed or occupied rental units.</t>
         </is>
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>Keep as the primary rent series.</t>
+          <t>Retain as multifamily supply proxy.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>rent growth MoM</t>
+          <t>price-to-rent</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Renter</t>
+          <t>Overall housing market</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -1881,7 +1849,7 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Zillow ZORI</t>
+          <t>Zillow ZHVI and ZORI</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -1889,7 +1857,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F20" s="5" t="inlineStr">
+      <c r="F20" s="4" t="inlineStr">
         <is>
           <t>Constructed variable</t>
         </is>
@@ -1901,7 +1869,7 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>zori_growth_mom</t>
+          <t>price_to_rent_ratio</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
@@ -1916,7 +1884,7 @@
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>2015-02-28</t>
+          <t>2015-01-31</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
@@ -1926,24 +1894,24 @@
       </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>Depends on the active smoothed seasonally adjusted ZORI vintage.</t>
+          <t>Index-based valuation ratio.</t>
         </is>
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>Retain as a constructed series.</t>
+          <t>Keep explicit formula.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>rent growth YoY</t>
+          <t>inventory-to-sales</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Renter</t>
+          <t>Overall housing market</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -1953,7 +1921,7 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Zillow ZORI</t>
+          <t>Redfin Data Center</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
@@ -1961,7 +1929,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F21" s="5" t="inlineStr">
+      <c r="F21" s="4" t="inlineStr">
         <is>
           <t>Constructed variable</t>
         </is>
@@ -1973,7 +1941,7 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>zori_growth_yoy</t>
+          <t>inventory_to_sales_ratio|sales_to_inventory_ratio</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
@@ -1988,7 +1956,7 @@
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>2016-01-31</t>
+          <t>2012-01-31</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr">
@@ -1998,90 +1966,106 @@
       </c>
       <c r="M21" s="2" t="inlineStr">
         <is>
-          <t>Requires twelve-month continuity in the active ZORI vintage.</t>
+          <t>Uses for-sale inventory and sales, not total housing stock.</t>
         </is>
       </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t>Retain as a constructed series.</t>
+          <t>Keep both orientations clearly named.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>rental inventory</t>
+          <t>market tightness</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Renter</t>
+          <t>Overall housing market</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Supply</t>
+          <t>Constructed indicator</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>No verified official public source</t>
+          <t>Redfin Data Center</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F22" s="6" t="inlineStr">
-        <is>
-          <t>Missing — no verified public source</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="inlineStr"/>
-      <c r="H22" s="2" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>Constructed variable</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>analytics.county_monthly_panel</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>market_tightness_index|market_tightness_components</t>
+        </is>
+      </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>monthly</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>Los Angeles County or ZIPs</t>
-        </is>
-      </c>
-      <c r="K22" s="2" t="inlineStr"/>
-      <c r="L22" s="2" t="inlineStr"/>
+          <t>Los Angeles County</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>2012-01-31</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
       <c r="M22" s="2" t="inlineStr">
         <is>
-          <t>ZORI measures rent levels and cannot serve as rental inventory; no defensible official public listing-inventory series is verified.</t>
+          <t>Composite, not official provider statistic.</t>
         </is>
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>Leave unavailable until a documented public source with stable geography and methodology is found.</t>
+          <t>Retain component-count metadata.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>rental vacancy</t>
+          <t>affordability metrics</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Renter</t>
+          <t>Overall housing market</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Supply</t>
+          <t>Affordability</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>U.S. Census Housing Vacancy Survey</t>
+          <t>Zillow, Redfin, Freddie Mac</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -2096,64 +2080,64 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>analytics.state_quarterly_panel|analytics.metro_quarterly_panel</t>
+          <t>analytics.county_monthly_panel</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>hvs_rental_vacancy_rate_ca|hvs_rental_vacancy_rate_la_metro</t>
+          <t>price_to_rent_ratio|mortgage_payment_to_rent_10pct_down|mortgage_payment_to_rent_20pct_down</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>quarterly</t>
+          <t>monthly</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>Published state and/or metro geographies only</t>
+          <t>Los Angeles County</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>2005-03-31</t>
+          <t>2015-01-31</t>
         </is>
       </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="M23" s="2" t="inlineStr">
         <is>
-          <t>Los Angeles County is not an HVS published geography; sampling uncertainty must be retained.</t>
+          <t>Income-based ratios are deferred at this active stage.</t>
         </is>
       </c>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t>Retain at native frequency and rebuild through the pipeline.</t>
+          <t>Do not expose ACS-derived affordability columns until requested.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>multifamily permits</t>
+          <t>LAUS unemployment rate</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Renter</t>
+          <t>Macro</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Supply</t>
+          <t>Control</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>U.S. Census Building Permits Survey</t>
+          <t>BLS LAUS</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -2173,7 +2157,7 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>permits_5_plus_units</t>
+          <t>unemployment_rate</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
@@ -2188,7 +2172,7 @@
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>2000-01-31</t>
+          <t>1990-01-31</t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr">
@@ -2198,34 +2182,34 @@
       </c>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>Permits are authorizations and do not measure occupied or completed rental units.</t>
+          <t>County series is not seasonally adjusted and may be revised.</t>
         </is>
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>Retain the existing permits series and its status fields.</t>
+          <t>Archive API responses.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>renter household counts</t>
+          <t>LAUS labor force</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Renter</t>
+          <t>Macro</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Demographic</t>
+          <t>Control</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>ACS 5-year</t>
+          <t>BLS LAUS</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -2240,64 +2224,64 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>analytics.county_annual_structural|analytics.zcta_annual_structural</t>
+          <t>analytics.county_monthly_panel</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>acs_households</t>
+          <t>labor_force</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>annual 5-year estimate</t>
+          <t>monthly</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>Los Angeles County and ZCTAs</t>
+          <t>Los Angeles County</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>2024-12-31</t>
+          <t>1990-01-31</t>
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>2024-12-31</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="M25" s="2" t="inlineStr">
         <is>
-          <t>ACS 5-year estimates represent pooled survey periods and include margins of error.</t>
+          <t>County series is not seasonally adjusted and may be revised.</t>
         </is>
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>Retain at native frequency and rebuild through the pipeline.</t>
+          <t>Archive API responses.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>renter-occupied units</t>
+          <t>CES payroll employment</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Renter</t>
+          <t>Macro</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Demographic</t>
+          <t>Control</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>ACS 5-year</t>
+          <t>BLS CES</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -2312,64 +2296,64 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>analytics.county_annual_structural|analytics.zcta_annual_structural</t>
+          <t>analytics.metro_monthly_controls</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>acs_renter_occupied_units</t>
+          <t>ces_total_nonfarm_employment_sa</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>annual 5-year estimate</t>
+          <t>monthly</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>Los Angeles County and ZCTAs</t>
+          <t>Los Angeles metro</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>2024-12-31</t>
+          <t>2005-01-31</t>
         </is>
       </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t>2024-12-31</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="M26" s="2" t="inlineStr">
         <is>
-          <t>ACS 5-year estimates are not point-in-time monthly counts.</t>
+          <t>Metro establishment series; not county LAUS employment.</t>
         </is>
       </c>
       <c r="N26" s="2" t="inlineStr">
         <is>
-          <t>Retain at native frequency and rebuild through the pipeline.</t>
+          <t>Retain geography label.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>rent-to-income</t>
+          <t>personal income</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Renter</t>
+          <t>Macro</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Affordability</t>
+          <t>Control</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>ACS 5-year</t>
+          <t>BEA</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -2377,127 +2361,143 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F27" s="5" t="inlineStr">
-        <is>
-          <t>Constructed variable</t>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>analytics.county_annual_structural|analytics.zcta_annual_structural</t>
+          <t>analytics.state_quarterly_panel|analytics.county_annual_controls</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>annual_rent_to_income_ratio</t>
+          <t>bea_ca_personal_income_q_sa|bea_la_county_personal_income_annual</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>annual 5-year estimate</t>
+          <t>quarterly and annual</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>Los Angeles County and ZCTAs</t>
+          <t>California and Los Angeles County</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>2024-12-31</t>
+          <t>1948-03-31</t>
         </is>
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>2024-12-31</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="M27" s="2" t="inlineStr">
         <is>
-          <t>Annual estimate; monthly interpolation would create false precision.</t>
+          <t>State quarterly and county annual products differ.</t>
         </is>
       </c>
       <c r="N27" s="2" t="inlineStr">
         <is>
-          <t>Retain at native frequency and rebuild through the pipeline.</t>
+          <t>Retain native frequency.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>occupied-apartment growth</t>
+          <t>CPI / inflation</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Renter</t>
+          <t>Macro</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Outcome</t>
+          <t>Control</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>No verified exact public series</t>
+          <t>BLS CPI</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F28" s="7" t="inlineStr">
-        <is>
-          <t>Proxy only</t>
-        </is>
-      </c>
-      <c r="G28" s="2" t="inlineStr"/>
-      <c r="H28" s="2" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>analytics.metro_monthly_controls</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>cpi_u_all_items_la_nsa|cpi_inflation_yoy</t>
+        </is>
+      </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>annual at best</t>
+          <t>monthly with historical gaps</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>Los Angeles County or metro</t>
-        </is>
-      </c>
-      <c r="K28" s="2" t="inlineStr"/>
-      <c r="L28" s="2" t="inlineStr"/>
+          <t>Los Angeles published area</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>1914-12-31</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
       <c r="M28" s="2" t="inlineStr">
         <is>
-          <t>ACS renter-occupied units are broader than apartments and cannot be relabeled as occupied-apartment growth.</t>
+          <t>Local CPI is not seasonally adjusted and has historical publication gaps.</t>
         </is>
       </c>
       <c r="N28" s="2" t="inlineStr">
         <is>
-          <t>If used, label annual renter-occupied-unit growth explicitly as a proxy.</t>
+          <t>Preserve gaps.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>price-to-rent</t>
+          <t>price-to-income</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Overall housing market</t>
+          <t>Homeowner</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Constructed indicator</t>
+          <t>Affordability</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Zillow ZHVI and ZORI</t>
+          <t>ACS or BEA</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -2505,1118 +2505,38 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="F29" s="5" t="inlineStr">
-        <is>
-          <t>Constructed variable</t>
-        </is>
-      </c>
-      <c r="G29" s="2" t="inlineStr">
-        <is>
-          <t>analytics.county_monthly_panel</t>
-        </is>
-      </c>
-      <c r="H29" s="2" t="inlineStr">
-        <is>
-          <t>price_to_rent_ratio</t>
-        </is>
-      </c>
+      <c r="F29" s="6" t="inlineStr">
+        <is>
+          <t>Deferred</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr"/>
+      <c r="H29" s="2" t="inlineStr"/>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>monthly</t>
+          <t>annual or mixed</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>Los Angeles County</t>
-        </is>
-      </c>
-      <c r="K29" s="2" t="inlineStr">
-        <is>
-          <t>2015-01-31</t>
-        </is>
-      </c>
-      <c r="L29" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-31</t>
-        </is>
-      </c>
+          <t>Los Angeles County or ZIP</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr"/>
+      <c r="L29" s="2" t="inlineStr"/>
       <c r="M29" s="2" t="inlineStr">
         <is>
-          <t>Index-based valuation ratio rather than a transaction cap-rate measure.</t>
+          <t>Not part of the current active available-variable set.</t>
         </is>
       </c>
       <c r="N29" s="2" t="inlineStr">
         <is>
-          <t>Retain the explicit ZHVI divided by annualized ZORI definition.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>inventory-to-sales</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>Overall housing market</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>Constructed indicator</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
-          <t>Redfin Data Center</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F30" s="5" t="inlineStr">
-        <is>
-          <t>Constructed variable</t>
-        </is>
-      </c>
-      <c r="G30" s="2" t="inlineStr">
-        <is>
-          <t>analytics.county_monthly_panel</t>
-        </is>
-      </c>
-      <c r="H30" s="2" t="inlineStr">
-        <is>
-          <t>inventory_to_sales_ratio</t>
-        </is>
-      </c>
-      <c r="I30" s="2" t="inlineStr">
-        <is>
-          <t>monthly</t>
-        </is>
-      </c>
-      <c r="J30" s="2" t="inlineStr">
-        <is>
-          <t>Los Angeles County</t>
-        </is>
-      </c>
-      <c r="K30" s="2" t="inlineStr">
-        <is>
-          <t>2012-01-31</t>
-        </is>
-      </c>
-      <c r="L30" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-31</t>
-        </is>
-      </c>
-      <c r="M30" s="2" t="inlineStr">
-        <is>
-          <t>This is inventory divided by monthly sales and is not housing-stock turnover.</t>
-        </is>
-      </c>
-      <c r="N30" s="2" t="inlineStr">
-        <is>
-          <t>Retain for compatibility and add the clearly directed sales_to_inventory_ratio.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>housing turnover</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>Overall housing market</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="inlineStr">
-        <is>
-          <t>Constructed indicator</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="inlineStr">
-        <is>
-          <t>Redfin homes sold and ACS housing stock</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F31" s="5" t="inlineStr">
-        <is>
-          <t>Constructed variable</t>
-        </is>
-      </c>
-      <c r="G31" s="2" t="inlineStr">
-        <is>
-          <t>analytics.county_annual_structural</t>
-        </is>
-      </c>
-      <c r="H31" s="2" t="inlineStr">
-        <is>
-          <t>sales_to_housing_stock_turnover</t>
-        </is>
-      </c>
-      <c r="I31" s="2" t="inlineStr">
-        <is>
-          <t>monthly numerator and annual denominator</t>
-        </is>
-      </c>
-      <c r="J31" s="2" t="inlineStr">
-        <is>
-          <t>Los Angeles County</t>
-        </is>
-      </c>
-      <c r="K31" s="2" t="inlineStr">
-        <is>
-          <t>2024-12-31</t>
-        </is>
-      </c>
-      <c r="L31" s="2" t="inlineStr">
-        <is>
-          <t>2024-12-31</t>
-        </is>
-      </c>
-      <c r="M31" s="2" t="inlineStr">
-        <is>
-          <t>Housing-stock denominator is missing and must remain annual.</t>
-        </is>
-      </c>
-      <c r="N31" s="2" t="inlineStr">
-        <is>
-          <t>Retain at native frequency and rebuild through the pipeline.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>market tightness</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>Overall housing market</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>Constructed indicator</t>
-        </is>
-      </c>
-      <c r="D32" s="2" t="inlineStr">
-        <is>
-          <t>Redfin Data Center</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F32" s="5" t="inlineStr">
-        <is>
-          <t>Constructed variable</t>
-        </is>
-      </c>
-      <c r="G32" s="2" t="inlineStr">
-        <is>
-          <t>analytics.county_monthly_panel</t>
-        </is>
-      </c>
-      <c r="H32" s="2" t="inlineStr">
-        <is>
-          <t>market_tightness_index</t>
-        </is>
-      </c>
-      <c r="I32" s="2" t="inlineStr">
-        <is>
-          <t>monthly</t>
-        </is>
-      </c>
-      <c r="J32" s="2" t="inlineStr">
-        <is>
-          <t>Los Angeles County</t>
-        </is>
-      </c>
-      <c r="K32" s="2" t="inlineStr">
-        <is>
-          <t>2012-01-31</t>
-        </is>
-      </c>
-      <c r="L32" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-31</t>
-        </is>
-      </c>
-      <c r="M32" s="2" t="inlineStr">
-        <is>
-          <t>Composite depends on available components and is not an official provider statistic.</t>
-        </is>
-      </c>
-      <c r="N32" s="2" t="inlineStr">
-        <is>
-          <t>Retain component-count metadata and document the formula.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>market time</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>Overall housing market</t>
-        </is>
-      </c>
-      <c r="C33" s="2" t="inlineStr">
-        <is>
-          <t>Predictor</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>Redfin Data Center</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F33" s="3" t="inlineStr">
-        <is>
-          <t>Implemented</t>
-        </is>
-      </c>
-      <c r="G33" s="2" t="inlineStr">
-        <is>
-          <t>analytics.county_monthly_panel</t>
-        </is>
-      </c>
-      <c r="H33" s="2" t="inlineStr">
-        <is>
-          <t>days_on_market</t>
-        </is>
-      </c>
-      <c r="I33" s="2" t="inlineStr">
-        <is>
-          <t>monthly</t>
-        </is>
-      </c>
-      <c r="J33" s="2" t="inlineStr">
-        <is>
-          <t>Los Angeles County</t>
-        </is>
-      </c>
-      <c r="K33" s="2" t="inlineStr">
-        <is>
-          <t>2012-01-31</t>
-        </is>
-      </c>
-      <c r="L33" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-31</t>
-        </is>
-      </c>
-      <c r="M33" s="2" t="inlineStr">
-        <is>
-          <t>Provider median and not additive.</t>
-        </is>
-      </c>
-      <c r="N33" s="2" t="inlineStr">
-        <is>
-          <t>Expose in the overall-market view.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>price-drop share</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>Overall housing market</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>Leading indicator</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>Redfin Data Center</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F34" s="3" t="inlineStr">
-        <is>
-          <t>Implemented</t>
-        </is>
-      </c>
-      <c r="G34" s="2" t="inlineStr">
-        <is>
-          <t>analytics.county_monthly_panel</t>
-        </is>
-      </c>
-      <c r="H34" s="2" t="inlineStr">
-        <is>
-          <t>price_drop_share</t>
-        </is>
-      </c>
-      <c r="I34" s="2" t="inlineStr">
-        <is>
-          <t>monthly</t>
-        </is>
-      </c>
-      <c r="J34" s="2" t="inlineStr">
-        <is>
-          <t>Los Angeles County</t>
-        </is>
-      </c>
-      <c r="K34" s="2" t="inlineStr">
-        <is>
-          <t>2012-01-31</t>
-        </is>
-      </c>
-      <c r="L34" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-31</t>
-        </is>
-      </c>
-      <c r="M34" s="2" t="inlineStr">
-        <is>
-          <t>One source month is null; not equivalent to a count of listings.</t>
-        </is>
-      </c>
-      <c r="N34" s="2" t="inlineStr">
-        <is>
-          <t>Expose in the overall-market view.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>affordability metrics</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t>Overall housing market</t>
-        </is>
-      </c>
-      <c r="C35" s="2" t="inlineStr">
-        <is>
-          <t>Affordability</t>
-        </is>
-      </c>
-      <c r="D35" s="2" t="inlineStr">
-        <is>
-          <t>Zillow, Redfin, Freddie Mac, ACS, BEA</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F35" s="3" t="inlineStr">
-        <is>
-          <t>Implemented</t>
-        </is>
-      </c>
-      <c r="G35" s="2" t="inlineStr">
-        <is>
-          <t>analytics.county_monthly_panel|analytics.county_annual_structural</t>
-        </is>
-      </c>
-      <c r="H35" s="2" t="inlineStr">
-        <is>
-          <t>price_to_rent_ratio|mortgage_payment_to_rent_10pct_down|mortgage_payment_to_rent_20pct_down|annual_price_to_income_ratio|annual_rent_to_income_ratio</t>
-        </is>
-      </c>
-      <c r="I35" s="2" t="inlineStr">
-        <is>
-          <t>mixed</t>
-        </is>
-      </c>
-      <c r="J35" s="2" t="inlineStr">
-        <is>
-          <t>Los Angeles County</t>
-        </is>
-      </c>
-      <c r="K35" s="2" t="inlineStr">
-        <is>
-          <t>2015-01-31</t>
-        </is>
-      </c>
-      <c r="L35" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-31</t>
-        </is>
-      </c>
-      <c r="M35" s="2" t="inlineStr">
-        <is>
-          <t>Rent- and payment-based metrics exist; income-based annual metrics are missing.</t>
-        </is>
-      </c>
-      <c r="N35" s="2" t="inlineStr">
-        <is>
-          <t>Add annual price-to-income and rent-to-income after official income data is loaded.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>LAUS unemployment rate</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>Macro</t>
-        </is>
-      </c>
-      <c r="C36" s="2" t="inlineStr">
-        <is>
-          <t>Control</t>
-        </is>
-      </c>
-      <c r="D36" s="2" t="inlineStr">
-        <is>
-          <t>BLS LAUS</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F36" s="3" t="inlineStr">
-        <is>
-          <t>Implemented</t>
-        </is>
-      </c>
-      <c r="G36" s="2" t="inlineStr">
-        <is>
-          <t>analytics.county_monthly_panel</t>
-        </is>
-      </c>
-      <c r="H36" s="2" t="inlineStr">
-        <is>
-          <t>unemployment_rate</t>
-        </is>
-      </c>
-      <c r="I36" s="2" t="inlineStr">
-        <is>
-          <t>monthly</t>
-        </is>
-      </c>
-      <c r="J36" s="2" t="inlineStr">
-        <is>
-          <t>Los Angeles County</t>
-        </is>
-      </c>
-      <c r="K36" s="2" t="inlineStr">
-        <is>
-          <t>1990-01-31</t>
-        </is>
-      </c>
-      <c r="L36" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-31</t>
-        </is>
-      </c>
-      <c r="M36" s="2" t="inlineStr">
-        <is>
-          <t>County series is not seasonally adjusted and may be revised.</t>
-        </is>
-      </c>
-      <c r="N36" s="2" t="inlineStr">
-        <is>
-          <t>Retain immutable API responses and county geography.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>LAUS employment</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="inlineStr">
-        <is>
-          <t>Macro</t>
-        </is>
-      </c>
-      <c r="C37" s="2" t="inlineStr">
-        <is>
-          <t>Control</t>
-        </is>
-      </c>
-      <c r="D37" s="2" t="inlineStr">
-        <is>
-          <t>BLS LAUS</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F37" s="3" t="inlineStr">
-        <is>
-          <t>Implemented</t>
-        </is>
-      </c>
-      <c r="G37" s="2" t="inlineStr">
-        <is>
-          <t>analytics.county_monthly_panel</t>
-        </is>
-      </c>
-      <c r="H37" s="2" t="inlineStr">
-        <is>
-          <t>employment</t>
-        </is>
-      </c>
-      <c r="I37" s="2" t="inlineStr">
-        <is>
-          <t>monthly</t>
-        </is>
-      </c>
-      <c r="J37" s="2" t="inlineStr">
-        <is>
-          <t>Los Angeles County</t>
-        </is>
-      </c>
-      <c r="K37" s="2" t="inlineStr">
-        <is>
-          <t>1990-01-31</t>
-        </is>
-      </c>
-      <c r="L37" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-31</t>
-        </is>
-      </c>
-      <c r="M37" s="2" t="inlineStr">
-        <is>
-          <t>County series is not seasonally adjusted and differs conceptually from CES payroll employment.</t>
-        </is>
-      </c>
-      <c r="N37" s="2" t="inlineStr">
-        <is>
-          <t>Retain as a residence-based labor-market control.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>LAUS unemployment</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>Macro</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t>Control</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t>BLS LAUS</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F38" s="3" t="inlineStr">
-        <is>
-          <t>Implemented</t>
-        </is>
-      </c>
-      <c r="G38" s="2" t="inlineStr">
-        <is>
-          <t>analytics.county_monthly_panel</t>
-        </is>
-      </c>
-      <c r="H38" s="2" t="inlineStr">
-        <is>
-          <t>unemployment</t>
-        </is>
-      </c>
-      <c r="I38" s="2" t="inlineStr">
-        <is>
-          <t>monthly</t>
-        </is>
-      </c>
-      <c r="J38" s="2" t="inlineStr">
-        <is>
-          <t>Los Angeles County</t>
-        </is>
-      </c>
-      <c r="K38" s="2" t="inlineStr">
-        <is>
-          <t>1990-01-31</t>
-        </is>
-      </c>
-      <c r="L38" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-31</t>
-        </is>
-      </c>
-      <c r="M38" s="2" t="inlineStr">
-        <is>
-          <t>County series is not seasonally adjusted and may be revised.</t>
-        </is>
-      </c>
-      <c r="N38" s="2" t="inlineStr">
-        <is>
-          <t>Retain immutable API responses and county geography.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr">
-        <is>
-          <t>LAUS labor force</t>
-        </is>
-      </c>
-      <c r="B39" s="2" t="inlineStr">
-        <is>
-          <t>Macro</t>
-        </is>
-      </c>
-      <c r="C39" s="2" t="inlineStr">
-        <is>
-          <t>Control</t>
-        </is>
-      </c>
-      <c r="D39" s="2" t="inlineStr">
-        <is>
-          <t>BLS LAUS</t>
-        </is>
-      </c>
-      <c r="E39" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F39" s="3" t="inlineStr">
-        <is>
-          <t>Implemented</t>
-        </is>
-      </c>
-      <c r="G39" s="2" t="inlineStr">
-        <is>
-          <t>analytics.county_monthly_panel</t>
-        </is>
-      </c>
-      <c r="H39" s="2" t="inlineStr">
-        <is>
-          <t>labor_force</t>
-        </is>
-      </c>
-      <c r="I39" s="2" t="inlineStr">
-        <is>
-          <t>monthly</t>
-        </is>
-      </c>
-      <c r="J39" s="2" t="inlineStr">
-        <is>
-          <t>Los Angeles County</t>
-        </is>
-      </c>
-      <c r="K39" s="2" t="inlineStr">
-        <is>
-          <t>1990-01-31</t>
-        </is>
-      </c>
-      <c r="L39" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-31</t>
-        </is>
-      </c>
-      <c r="M39" s="2" t="inlineStr">
-        <is>
-          <t>County series is not seasonally adjusted and may be revised.</t>
-        </is>
-      </c>
-      <c r="N39" s="2" t="inlineStr">
-        <is>
-          <t>Retain immutable API responses and county geography.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>CES payroll employment</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="inlineStr">
-        <is>
-          <t>Macro</t>
-        </is>
-      </c>
-      <c r="C40" s="2" t="inlineStr">
-        <is>
-          <t>Control</t>
-        </is>
-      </c>
-      <c r="D40" s="2" t="inlineStr">
-        <is>
-          <t>BLS CES</t>
-        </is>
-      </c>
-      <c r="E40" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F40" s="3" t="inlineStr">
-        <is>
-          <t>Implemented</t>
-        </is>
-      </c>
-      <c r="G40" s="2" t="inlineStr">
-        <is>
-          <t>analytics.metro_monthly_controls</t>
-        </is>
-      </c>
-      <c r="H40" s="2" t="inlineStr">
-        <is>
-          <t>ces_total_nonfarm_employment_sa</t>
-        </is>
-      </c>
-      <c r="I40" s="2" t="inlineStr">
-        <is>
-          <t>monthly</t>
-        </is>
-      </c>
-      <c r="J40" s="2" t="inlineStr">
-        <is>
-          <t>Los Angeles-Long Beach-Anaheim MSA</t>
-        </is>
-      </c>
-      <c r="K40" s="2" t="inlineStr">
-        <is>
-          <t>2005-01-31</t>
-        </is>
-      </c>
-      <c r="L40" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-31</t>
-        </is>
-      </c>
-      <c r="M40" s="2" t="inlineStr">
-        <is>
-          <t>Establishment-based metro series must not be labeled as county employment.</t>
-        </is>
-      </c>
-      <c r="N40" s="2" t="inlineStr">
-        <is>
-          <t>Retain at native frequency and rebuild through the pipeline.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr">
-        <is>
-          <t>personal income</t>
-        </is>
-      </c>
-      <c r="B41" s="2" t="inlineStr">
-        <is>
-          <t>Macro</t>
-        </is>
-      </c>
-      <c r="C41" s="2" t="inlineStr">
-        <is>
-          <t>Control</t>
-        </is>
-      </c>
-      <c r="D41" s="2" t="inlineStr">
-        <is>
-          <t>Bureau of Economic Analysis</t>
-        </is>
-      </c>
-      <c r="E41" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F41" s="3" t="inlineStr">
-        <is>
-          <t>Implemented</t>
-        </is>
-      </c>
-      <c r="G41" s="2" t="inlineStr">
-        <is>
-          <t>analytics.state_quarterly_panel|analytics.county_annual_structural</t>
-        </is>
-      </c>
-      <c r="H41" s="2" t="inlineStr">
-        <is>
-          <t>bea_ca_personal_income_q_sa|bea_la_county_personal_income_annual</t>
-        </is>
-      </c>
-      <c r="I41" s="2" t="inlineStr">
-        <is>
-          <t>quarterly and annual</t>
-        </is>
-      </c>
-      <c r="J41" s="2" t="inlineStr">
-        <is>
-          <t>California and Los Angeles County</t>
-        </is>
-      </c>
-      <c r="K41" s="2" t="inlineStr">
-        <is>
-          <t>1948-03-31</t>
-        </is>
-      </c>
-      <c r="L41" s="2" t="inlineStr">
-        <is>
-          <t>2026-03-31</t>
-        </is>
-      </c>
-      <c r="M41" s="2" t="inlineStr">
-        <is>
-          <t>State quarterly and county annual products have different frequencies and units.</t>
-        </is>
-      </c>
-      <c r="N41" s="2" t="inlineStr">
-        <is>
-          <t>Retain at native frequency and rebuild through the pipeline.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>CPI / inflation</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>Macro</t>
-        </is>
-      </c>
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t>Control</t>
-        </is>
-      </c>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
-          <t>BLS CPI</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F42" s="3" t="inlineStr">
-        <is>
-          <t>Implemented</t>
-        </is>
-      </c>
-      <c r="G42" s="2" t="inlineStr">
-        <is>
-          <t>analytics.metro_monthly_controls</t>
-        </is>
-      </c>
-      <c r="H42" s="2" t="inlineStr">
-        <is>
-          <t>cpi_u_all_items_la_nsa|cpi_inflation_yoy</t>
-        </is>
-      </c>
-      <c r="I42" s="2" t="inlineStr">
-        <is>
-          <t>published monthly with historical frequency gaps</t>
-        </is>
-      </c>
-      <c r="J42" s="2" t="inlineStr">
-        <is>
-          <t>Los Angeles published area</t>
-        </is>
-      </c>
-      <c r="K42" s="2" t="inlineStr">
-        <is>
-          <t>1914-12-31</t>
-        </is>
-      </c>
-      <c r="L42" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-31</t>
-        </is>
-      </c>
-      <c r="M42" s="2" t="inlineStr">
-        <is>
-          <t>Local CPI is not seasonally adjusted and historical publication gaps must remain visible.</t>
-        </is>
-      </c>
-      <c r="N42" s="2" t="inlineStr">
-        <is>
-          <t>Retain at native frequency and rebuild through the pipeline.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="2" t="inlineStr">
-        <is>
-          <t>mortgage rate</t>
-        </is>
-      </c>
-      <c r="B43" s="2" t="inlineStr">
-        <is>
-          <t>Macro</t>
-        </is>
-      </c>
-      <c r="C43" s="2" t="inlineStr">
-        <is>
-          <t>Control</t>
-        </is>
-      </c>
-      <c r="D43" s="2" t="inlineStr">
-        <is>
-          <t>Freddie Mac PMMS</t>
-        </is>
-      </c>
-      <c r="E43" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F43" s="3" t="inlineStr">
-        <is>
-          <t>Implemented</t>
-        </is>
-      </c>
-      <c r="G43" s="2" t="inlineStr">
-        <is>
-          <t>analytics.county_monthly_panel</t>
-        </is>
-      </c>
-      <c r="H43" s="2" t="inlineStr">
-        <is>
-          <t>mortgage_rate_30y_monthly_average</t>
-        </is>
-      </c>
-      <c r="I43" s="2" t="inlineStr">
-        <is>
-          <t>weekly aggregated to monthly</t>
-        </is>
-      </c>
-      <c r="J43" s="2" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="K43" s="2" t="inlineStr">
-        <is>
-          <t>1971-04-02</t>
-        </is>
-      </c>
-      <c r="L43" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-25</t>
-        </is>
-      </c>
-      <c r="M43" s="2" t="inlineStr">
-        <is>
-          <t>National rather than local; monthly value is a transparent aggregation of weekly observations.</t>
-        </is>
-      </c>
-      <c r="N43" s="2" t="inlineStr">
-        <is>
-          <t>Expose with U.S. geography in the macro-controls view.</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>Treasury rate and mortgage spread</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="inlineStr">
-        <is>
-          <t>Macro</t>
-        </is>
-      </c>
-      <c r="C44" s="2" t="inlineStr">
-        <is>
-          <t>Control</t>
-        </is>
-      </c>
-      <c r="D44" s="2" t="inlineStr">
-        <is>
-          <t>U.S. Treasury or Federal Reserve</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F44" s="8" t="inlineStr">
-        <is>
-          <t>Deferred</t>
-        </is>
-      </c>
-      <c r="G44" s="2" t="inlineStr"/>
-      <c r="H44" s="2" t="inlineStr"/>
-      <c r="I44" s="2" t="inlineStr">
-        <is>
-          <t>daily or weekly</t>
-        </is>
-      </c>
-      <c r="J44" s="2" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="K44" s="2" t="inlineStr"/>
-      <c r="L44" s="2" t="inlineStr"/>
-      <c r="M44" s="2" t="inlineStr">
-        <is>
-          <t>Not present in the current project and explicitly optional under the requested scope.</t>
-        </is>
-      </c>
-      <c r="N44" s="2" t="inlineStr">
-        <is>
-          <t>Defer unless the project scope is expanded.</t>
+          <t>Add later only with an explicit denominator choice.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N44"/>
+  <autoFilter ref="A1:N29"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Implement ACS rental availability proxy
</commit_message>
<xml_diff>
--- a/metadata/data_gap_analysis.xlsx
+++ b/metadata/data_gap_analysis.xlsx
@@ -1519,37 +1519,37 @@
       <c r="I11" s="3" t="inlineStr"/>
       <c r="J11" s="6" t="inlineStr">
         <is>
-          <t>Partially implemented – active all-residential proxy only</t>
+          <t>Partially implemented – ACS annual availability and HUD/USPS quarterly proxies; monthly listings unavailable</t>
         </is>
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
-          <t>hud_usps_ncwm_quarterly</t>
+          <t>census_acs_5year_b25003|census_acs_5year_b25004|hud_usps_ncwm_quarterly</t>
         </is>
       </c>
       <c r="L11" s="4" t="inlineStr">
         <is>
-          <t>usps_total_residential_addresses|usps_short_term_vacant_residential_addresses|usps_long_term_vacant_residential_addresses|usps_vacant_residential_addresses|usps_no_stat_residential_addresses|usps_active_residential_addresses|usps_residential_vacancy_rate|usps_residential_no_stat_rate</t>
+          <t>acs_renter_occupied_units|acs_renter_occupied_units_moe|acs_for_rent_vacant_units|acs_for_rent_vacant_units_moe|acs_rental_availability_rate|usps_total_residential_addresses|usps_short_term_vacant_residential_addresses|usps_long_term_vacant_residential_addresses|usps_vacant_residential_addresses|usps_no_stat_residential_addresses|usps_active_residential_addresses|usps_residential_vacancy_rate|usps_residential_no_stat_rate</t>
         </is>
       </c>
       <c r="M11" s="3" t="inlineStr">
         <is>
-          <t>analytics.fact_housing_observation|data/restricted/hud_usps/active/ca_county_quarterly.parquet|data/restricted/hud_usps/active/la_tract_2020_quarterly.parquet|data/restricted/hud_usps/active/la_postal_zip_county_part_quarterly.parquet|data/restricted/hud_usps/active/long_observations_with_lineage.parquet</t>
+          <t>analytics.fact_housing_observation|analytics.county_annual_controls|data/restricted/hud_usps/active/ca_county_quarterly.parquet|data/restricted/hud_usps/active/la_tract_2020_quarterly.parquet|data/restricted/hud_usps/active/la_postal_zip_county_part_quarterly.parquet|data/restricted/hud_usps/active/long_observations_with_lineage.parquet</t>
         </is>
       </c>
       <c r="N11" s="3" t="inlineStr">
         <is>
-          <t>usps_total_residential_addresses|usps_short_term_vacant_residential_addresses|usps_long_term_vacant_residential_addresses|usps_vacant_residential_addresses|usps_no_stat_residential_addresses|usps_active_residential_addresses|usps_residential_vacancy_rate|usps_residential_no_stat_rate</t>
+          <t>acs_renter_occupied_units|acs_renter_occupied_units_moe|acs_for_rent_vacant_units|acs_for_rent_vacant_units_moe|acs_rental_availability_rate|usps_total_residential_addresses|usps_short_term_vacant_residential_addresses|usps_long_term_vacant_residential_addresses|usps_vacant_residential_addresses|usps_no_stat_residential_addresses|usps_active_residential_addresses|usps_residential_vacancy_rate|usps_residential_no_stat_rate</t>
         </is>
       </c>
       <c r="O11" s="3" t="inlineStr">
         <is>
-          <t>active all-residential proxy</t>
+          <t>separate annual and quarterly proxies</t>
         </is>
       </c>
       <c r="P11" s="3" t="inlineStr">
         <is>
-          <t>The eight active HUD-USPS variables are native-quarterly only. The vacancy proxy is (short-term vacant + long-term vacant) / total residential addresses, while no-stat remains a separate diagnostic. Direct provider components are observed at standardized 2020-tract geography; California county aggregates are constructed, and Los Angeles County postal-ZIP county-parts are modeled with the fixed 2026 Q1 crosswalk. Detailed tract and modeled ZIP-part derivatives remain access-controlled under the HUD-USPS sublicense. This is not true rental-listing inventory; ZORI is not inventory (it is a rent index), and Redfin for-sale active listings are not a valid substitute. The former derived package file was deleted; its historical quarantine manifest is superseded and is not an active input.</t>
+          <t>The annual ACS rental-availability proxy is for-rent vacant units divided by renter-occupied plus for-rent vacant units, using matched B25003 and B25004 estimates. Component 90% margins of error are retained, and unreliable county ratios are suppressed. Direct ACS counts and margins of error are retained at county and ZCTA geography; ZCTAs are not postal ZIPs. The eight active HUD-USPS variables are native-quarterly only and remain a separate all-residential measure. The vacancy proxy is (short-term vacant + long-term vacant) / total residential addresses, while no-stat remains a separate diagnostic. Direct provider components are observed at standardized 2020-tract geography; California county aggregates are constructed, and Los Angeles County postal-ZIP county-parts are modeled with the fixed 2026 Q1 crosswalk. Detailed tract and modeled ZIP-part derivatives remain access-controlled under the HUD-USPS sublicense. This is not true rental-listing inventory; ZORI is not inventory (it is a rent index), and Redfin for-sale active listings are not a valid substitute. The monthly rental-listing series remains missing at documented source and license acquisition. The former derived package file was deleted; its historical quarantine manifest is superseded and is not an active input.</t>
         </is>
       </c>
       <c r="Q11" s="3" t="inlineStr"/>
@@ -1560,7 +1560,7 @@
         <v>1</v>
       </c>
       <c r="V11" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W11" s="3" t="b">
         <v>1</v>
@@ -1575,11 +1575,11 @@
         <v>46112</v>
       </c>
       <c r="AA11" s="3" t="n">
-        <v>1768936</v>
+        <v>1770036</v>
       </c>
       <c r="AB11" s="3" t="inlineStr">
         <is>
-          <t>9256 missing of 1768936 fact rows</t>
+          <t>9256 missing of 1770036 fact rows</t>
         </is>
       </c>
       <c r="AC11" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Use neutral environment and workbook labels
</commit_message>
<xml_diff>
--- a/metadata/data_gap_analysis.xlsx
+++ b/metadata/data_gap_analysis.xlsx
@@ -224,9 +224,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="ChatGPT">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Housing Database">
   <a:themeElements>
-    <a:clrScheme name="ChatGPT">
+    <a:clrScheme name="Housing Database">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -276,7 +276,7 @@
         <a:cs typeface="Calibri"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="ChatGPT">
+    <a:fmtScheme name="Housing Database">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>

</xml_diff>

<commit_message>
Publish current database, variable metadata and CSV browser
</commit_message>
<xml_diff>
--- a/metadata/data_gap_analysis.xlsx
+++ b/metadata/data_gap_analysis.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Gap Analysis" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Gap Analysis'!$A$1:$AC$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Gap Analysis'!$A$1:$AC$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -71,13 +71,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -445,24 +445,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC14"/>
+  <dimension ref="A1:AC11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="31" customWidth="1" min="1" max="1"/>
     <col width="42" customWidth="1" min="2" max="2"/>
     <col width="42" customWidth="1" min="3" max="3"/>
     <col width="39" customWidth="1" min="4" max="4"/>
     <col width="30" customWidth="1" min="5" max="5"/>
     <col width="36" customWidth="1" min="6" max="6"/>
-    <col width="35" customWidth="1" min="7" max="7"/>
+    <col width="27" customWidth="1" min="7" max="7"/>
     <col width="42" customWidth="1" min="8" max="8"/>
     <col width="42" customWidth="1" min="9" max="9"/>
-    <col width="42" customWidth="1" min="10" max="10"/>
+    <col width="39" customWidth="1" min="10" max="10"/>
     <col width="42" customWidth="1" min="11" max="11"/>
     <col width="42" customWidth="1" min="12" max="12"/>
     <col width="42" customWidth="1" min="13" max="13"/>
     <col width="42" customWidth="1" min="14" max="14"/>
-    <col width="40" customWidth="1" min="15" max="15"/>
+    <col width="42" customWidth="1" min="15" max="15"/>
     <col width="42" customWidth="1" min="16" max="16"/>
     <col width="18" customWidth="1" min="17" max="17"/>
     <col width="22" customWidth="1" min="18" max="18"/>
@@ -475,7 +475,7 @@
     <col width="21" customWidth="1" min="25" max="25"/>
     <col width="21" customWidth="1" min="26" max="26"/>
     <col width="12" customWidth="1" min="27" max="27"/>
-    <col width="35" customWidth="1" min="28" max="28"/>
+    <col width="33" customWidth="1" min="28" max="28"/>
     <col width="42" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
@@ -634,12 +634,12 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Homebuying Costs - Property Insurance</t>
+          <t>Aggregate Home Equity</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Homebuying Costs – Property Insurance</t>
+          <t>Aggregate Home Equity</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr"/>
@@ -648,31 +648,47 @@
       <c r="G2" s="3" t="inlineStr"/>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>NAIC only publishes state-level averages</t>
+          <t>No public state/county balance-sheet series; Fed Flow of Funds is national only</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>Use CA state series.</t>
-        </is>
-      </c>
-      <c r="J2" s="3" t="inlineStr">
-        <is>
-          <t>Not implemented</t>
-        </is>
-      </c>
-      <c r="K2" s="4" t="inlineStr"/>
-      <c r="L2" s="4" t="inlineStr"/>
-      <c r="M2" s="3" t="inlineStr"/>
-      <c r="N2" s="3" t="inlineStr"/>
+          <t>Use the Version A benchmark: published ACS B25082 aggregate owner values less the matched-universe, California-calibrated first-mortgage debt benchmark; add published mortgage-free owner value in full for all-owner equity.</t>
+        </is>
+      </c>
+      <c r="J2" s="4" t="inlineStr">
+        <is>
+          <t>Partially implemented</t>
+        </is>
+      </c>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>census_acs5_finance|census_acs5_pums_housing_ca|census_tract_to_puma_2010|census_tract_to_puma_2020|fhfa_nmdb_joint_distribution|fhfa_nmdb_ca_upb|freddie_mac_pmms|bls_cpi_u_us_city_average|census_sipp_2025_state_wealth_2024</t>
+        </is>
+      </c>
+      <c r="L2" s="5" t="inlineStr">
+        <is>
+          <t>acs_implied_owner_occupied_home_equity_mortgaged_pmms_20y_scenario_benchmark|acs_implied_owner_occupied_home_equity_mortgaged_pmms_25y_scenario_benchmark|acs_implied_owner_occupied_home_equity_mortgaged_pmms_30y_scenario_benchmark|acs_implied_owner_occupied_home_equity_all_pmms_20y_scenario_benchmark|acs_implied_owner_occupied_home_equity_all_pmms_25y_scenario_benchmark|acs_implied_owner_occupied_home_equity_all_pmms_30y_scenario_benchmark|acs_implied_owner_occupied_home_equity_mortgaged_benchmark|acs_implied_owner_occupied_home_equity_all_benchmark|acs_implied_owner_occupied_home_equity_mortgaged_real_2024_benchmark|acs_implied_owner_occupied_home_equity_all_real_2024_benchmark|sipp_ca_aggregate_positive_home_equity_sensitivity</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>analytics.housing_finance_benchmark|analytics.state_annual_controls</t>
+        </is>
+      </c>
+      <c r="N2" s="3" t="inlineStr">
+        <is>
+          <t>acs_implied_owner_occupied_home_equity_all_pmms_20y_scenario_benchmark|acs_implied_owner_occupied_home_equity_all_pmms_25y_scenario_benchmark|acs_implied_owner_occupied_home_equity_all_pmms_30y_scenario_benchmark|sipp_ca_aggregate_positive_home_equity_sensitivity</t>
+        </is>
+      </c>
       <c r="O2" s="3" t="inlineStr">
         <is>
-          <t>deferred</t>
+          <t>scenario sensitivity|published-table sensitivity|schema only</t>
         </is>
       </c>
       <c r="P2" s="3" t="inlineStr">
         <is>
-          <t>The sheet specifies a CA state NAIC series; NAIC/state homeowners-insurance data is not loaded yet.</t>
+          <t>The methodology-authorized raw PMMS 20/25/30-year debt sensitivities produce matching mortgaged-owner and all-owner equity scenarios for all 58 California counties. They are explicit uncalibrated scenarios. The official 2025 SIPP state wealth table now also produces one separately labeled 2024 California positive-home-equity sensitivity of $4,913,341,020,000 from rounded published inputs. It is conditional on positive equity, truncates the conditional mean to net worth below the 99th percentile, and has no valid covariance-based aggregate standard error. It is not the preferred matched-universe county equity target. The calibrated nominal and real equity targets remain null until an exact-date, owner-occupied first-lien California UPB control is available. The older B25106 midpoint proxy remains only as a separately labeled legacy modeled scenario.</t>
         </is>
       </c>
       <c r="Q2" s="3" t="inlineStr"/>
@@ -683,20 +699,28 @@
         <v>0</v>
       </c>
       <c r="V2" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W2" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X2" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y2" s="3" t="inlineStr"/>
-      <c r="Z2" s="3" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="Y2" s="6" t="n">
+        <v>45657</v>
+      </c>
+      <c r="Z2" s="6" t="n">
+        <v>45657</v>
+      </c>
       <c r="AA2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB2" s="3" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AB2" s="3" t="inlineStr">
+        <is>
+          <t>0 missing of 1 fact rows</t>
+        </is>
+      </c>
       <c r="AC2" s="3" t="inlineStr">
         <is>
           <t>Review documented limitation before modeling</t>
@@ -711,12 +735,12 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Rental price increase in non-rent-controlled locations</t>
+          <t>Aggregate Mortgage Debt (outstanding balances)</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Rental price increase in non–rent-controlled locations</t>
+          <t>Aggregate Mortgage Debt (outstanding balances)</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr"/>
@@ -725,47 +749,47 @@
       <c r="G3" s="3" t="inlineStr"/>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>Public rent indices do not flag rent-control status</t>
+          <t>ACS reports payments, not balances; no public CA/LA balance series</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>Use Zillow ZORI and exclude geographies by construction-year share (post-1995 / post-2005 proxy) or interact with policy exposure.</t>
-        </is>
-      </c>
-      <c r="J3" s="3" t="inlineStr">
-        <is>
-          <t>Not implemented</t>
-        </is>
-      </c>
-      <c r="K3" s="4" t="inlineStr">
-        <is>
-          <t>zillow_county_zori_smoothed_sa|zillow_zip_zori_smoothed_sa</t>
-        </is>
-      </c>
-      <c r="L3" s="4" t="inlineStr">
-        <is>
-          <t>zori_smoothed_sa</t>
+          <t>Use the Version A benchmark: direct ACS B25089/B25081 levels, weighted ACS PUMS first-mortgage P&amp;I parameters, an exact-date joint NMDB rate-term distribution, and a compatible California UPB control. Retain PMMS only as a labeled sensitivity fallback.</t>
+        </is>
+      </c>
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t>Partially implemented</t>
+        </is>
+      </c>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>census_acs5_finance|census_acs5_pums_housing_ca|census_tract_to_puma_2010|census_tract_to_puma_2020|fhfa_nmdb_joint_distribution|fhfa_nmdb_ca_upb|freddie_mac_pmms|census_sipp_2025_state_debt_2024|census_ahs_2023_ca_table14a</t>
+        </is>
+      </c>
+      <c r="L3" s="5" t="inlineStr">
+        <is>
+          <t>acs_implied_first_mortgage_balance_raw_pmms_20y_sensitivity_benchmark|acs_implied_first_mortgage_balance_raw_pmms_25y_sensitivity_benchmark|acs_implied_first_mortgage_balance_raw_pmms_30y_sensitivity_benchmark|acs_implied_first_mortgage_balance_raw_benchmark|acs_implied_first_mortgage_balance_cal_benchmark|acs_first_mortgage_debt_per_mortgaged_owner_unit_benchmark|acs_first_mortgage_debt_per_owner_unit_benchmark|acs_first_mortgage_debt_per_capita_benchmark|acs_first_mortgage_debt_to_owner_income_benchmark|sipp_ca_aggregate_primary_residence_debt_sensitivity|ahs_ca_reported_case_primary_mortgage_outstanding_principal_proxy</t>
         </is>
       </c>
       <c r="M3" s="3" t="inlineStr">
         <is>
-          <t>analytics.county_monthly_panel|analytics.zip_monthly_panel</t>
+          <t>analytics.housing_finance_benchmark|analytics.state_annual_controls</t>
         </is>
       </c>
       <c r="N3" s="3" t="inlineStr">
         <is>
-          <t>zori</t>
+          <t>acs_implied_first_mortgage_balance_cal_benchmark|sipp_ca_aggregate_primary_residence_debt_sensitivity|ahs_ca_reported_case_primary_mortgage_outstanding_principal_proxy</t>
         </is>
       </c>
       <c r="O3" s="3" t="inlineStr">
         <is>
-          <t>proxy input</t>
+          <t>scenario sensitivity|published-table sensitivity|reported-case public proxy|schema only</t>
         </is>
       </c>
       <c r="P3" s="3" t="inlineStr">
         <is>
-          <t>ZORI is loaded, but the sheet workaround also requires construction-year/rent-control exposure filters that are not implemented.</t>
+          <t>Version A publishes explicit raw PMMS 20/25/30-year debt sensitivities for all 58 California counties while retaining the composite raw envelope. The official 2025 SIPP state debt table adds a broader 2024 California Home Debt sensitivity of $1,627,458,504,000. The official 2023 California AHS Table 14A adds a reported-case primary-mortgage proxy of $1,413,679,720,000 from 3,381,200 reported-bin households times the $418,100 conditional mean. AHS excludes 1,203,800 regular-mortgage households with no reported balance (26.2540 percent), does not make a missing-at-random extrapolation, may not match legal first-lien status, and has no covariance-based aggregate uncertainty measure. Neither public sensitivity matches the current Version A target universe and 2022-07-01 reference date exactly. Calibrated debt and normalized ratios remain null; the older B25106 proxy remains a separate legacy construction.</t>
         </is>
       </c>
       <c r="Q3" s="3" t="inlineStr"/>
@@ -773,7 +797,7 @@
       <c r="S3" s="3" t="inlineStr"/>
       <c r="T3" s="3" t="inlineStr"/>
       <c r="U3" s="3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V3" s="3" t="b">
         <v>1</v>
@@ -784,18 +808,18 @@
       <c r="X3" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="Y3" s="5" t="n">
-        <v>42035</v>
-      </c>
-      <c r="Z3" s="5" t="n">
-        <v>46173</v>
+      <c r="Y3" s="6" t="n">
+        <v>45291</v>
+      </c>
+      <c r="Z3" s="6" t="n">
+        <v>45657</v>
       </c>
       <c r="AA3" s="3" t="n">
-        <v>33702</v>
+        <v>2</v>
       </c>
       <c r="AB3" s="3" t="inlineStr">
         <is>
-          <t>15699 missing of 33702 fact rows</t>
+          <t>0 missing of 2 fact rows</t>
         </is>
       </c>
       <c r="AC3" s="3" t="inlineStr">
@@ -812,12 +836,12 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>New Apartments Completed (county time series)</t>
+          <t>Rental price increase in non-rent-controlled locations</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>New Apartments Completed (county time series)</t>
+          <t>Rental price increase in non–rent-controlled locations</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr"/>
@@ -826,47 +850,47 @@
       <c r="G4" s="3" t="inlineStr"/>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>Clean completions data not consistently public at county level</t>
+          <t>Public rent indices do not flag rent-control status</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Proxy with lagged multifamily permits (5+) using completion lag structure; lags uncertain.</t>
-        </is>
-      </c>
-      <c r="J4" s="3" t="inlineStr">
-        <is>
-          <t>Proxy input only</t>
-        </is>
-      </c>
-      <c r="K4" s="4" t="inlineStr">
-        <is>
-          <t>census_bps_county|census_bps_state</t>
-        </is>
-      </c>
-      <c r="L4" s="4" t="inlineStr">
-        <is>
-          <t>permits_5_plus_units</t>
+          <t>Use Zillow ZORI with the methodology-listed ACS B25032/B25127 renter structure and year-built inputs. Preserve lower/upper structural exposure bounds because published ACS bins cannot recover an exact rolling 15-year cutoff; construct an exact point exposure only after a complete dated property-level policy and exemption crosswalk is available.</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>Partially implemented</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>zillow_county_zori_smoothed_sa|zillow_zip_zori_smoothed_sa|census_acs_5year_b25032|census_acs_5year_b25127</t>
+        </is>
+      </c>
+      <c r="L4" s="5" t="inlineStr">
+        <is>
+          <t>zori_smoothed_sa|acs_renter_occupied_1_unit_share|acs_renter_occupied_2_to_4_units_share|acs_renter_occupied_5_plus_units_share|acs_renter_occupied_mobile_other_share|acs_renter_recent_construction_share_lower_bound|acs_renter_recent_construction_share_upper_bound|noncontrolled_exposure_share_structural_proxy_lower_bound|noncontrolled_exposure_share_structural_proxy_upper_bound|exposure_adjusted_noncontrolled_rent_growth_structural_proxy_lower_bound|exposure_adjusted_noncontrolled_rent_growth_structural_proxy_upper_bound</t>
         </is>
       </c>
       <c r="M4" s="3" t="inlineStr">
         <is>
-          <t>analytics.fact_housing_observation|analytics.county_monthly_panel</t>
+          <t>analytics.county_monthly_panel|analytics.zip_monthly_panel|analytics.county_annual_controls|analytics.zcta_annual_controls</t>
         </is>
       </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
-          <t>permits_5_plus_units</t>
+          <t>noncontrolled_exposure_share_structural_proxy_lower_bound|noncontrolled_exposure_share_structural_proxy_upper_bound|exposure_adjusted_noncontrolled_rent_growth_structural_proxy_lower_bound|exposure_adjusted_noncontrolled_rent_growth_structural_proxy_upper_bound</t>
         </is>
       </c>
       <c r="O4" s="3" t="inlineStr">
         <is>
-          <t>proxy input</t>
+          <t>observed rent index|constructed structural proxy bounds|annual exposure-scaled sensitivity</t>
         </is>
       </c>
       <c r="P4" s="3" t="inlineStr">
         <is>
-          <t>The sheet workaround is lagged multifamily permits with an explicit completion-lag structure; permits are loaded, but no completion proxy is calculated.</t>
+          <t>The methodology-listed official ACS B25032/B25127 inputs and eight same-vintage annual structure/age/exposure constructions are implemented at county and Census-ZCTA geography; the structural exposure bounds are null before 2020 and are not legal eligibility determinations. Five 2020-2024 annual Los Angeles County sensitivities multiply the exact December county ZORI year-over-year change by the same-ending-year structural lower and upper exposure bounds without monthly carry-forward. These are not observed rent growth inside legally noncontrolled units. Exact noncontrolled_exposure_share and exact exposure-adjusted growth remain unavailable until a complete dated property-level policy/exemption crosswalk exists. The official-source scaffold is not applied, and Census ZCTAs are not USPS postal ZIPs.</t>
         </is>
       </c>
       <c r="Q4" s="3" t="inlineStr"/>
@@ -885,18 +909,18 @@
       <c r="X4" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="Y4" s="5" t="n">
-        <v>36556</v>
-      </c>
-      <c r="Z4" s="5" t="n">
-        <v>46173</v>
+      <c r="Y4" s="6" t="n">
+        <v>44196</v>
+      </c>
+      <c r="Z4" s="6" t="n">
+        <v>45657</v>
       </c>
       <c r="AA4" s="3" t="n">
-        <v>634</v>
+        <v>2760</v>
       </c>
       <c r="AB4" s="3" t="inlineStr">
         <is>
-          <t>0 missing of 634 fact rows</t>
+          <t>0 missing of 2760 panel cells</t>
         </is>
       </c>
       <c r="AC4" s="3" t="inlineStr">
@@ -913,12 +937,12 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Multifamily Under Construction</t>
+          <t>Eviction trends (high-frequency, consistent)</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Multifamily Under Construction</t>
+          <t>Eviction trends (high-frequency, consistent)</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr"/>
@@ -927,47 +951,47 @@
       <c r="G5" s="3" t="inlineStr"/>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>No public stock measure at county/state level</t>
+          <t>County coverage uneven; time consistency varies</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>Build pipeline stock: cumulative MF permits minus assumed completions over rolling window.</t>
-        </is>
-      </c>
-      <c r="J5" s="3" t="inlineStr">
-        <is>
-          <t>Proxy input only</t>
-        </is>
-      </c>
-      <c r="K5" s="4" t="inlineStr">
-        <is>
-          <t>census_bps_county|census_bps_state</t>
-        </is>
-      </c>
-      <c r="L5" s="4" t="inlineStr">
-        <is>
-          <t>permits_5_plus_units</t>
+          <t>Use Eviction Lab ETS only where the official release contains the geography; otherwise retain official annual modeled estimates at native annual frequency without interpolation.</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>Partially implemented</t>
+        </is>
+      </c>
+      <c r="K5" s="5" t="inlineStr">
+        <is>
+          <t>eviction_lab_county_estimates</t>
+        </is>
+      </c>
+      <c r="L5" s="5" t="inlineStr">
+        <is>
+          <t>eviction_lab_filings_estimate_annual|eviction_lab_filings_rate_estimate_annual|eviction_lab_households_threatened_estimate_annual|eviction_lab_households_threatened_rate_estimate_annual</t>
         </is>
       </c>
       <c r="M5" s="3" t="inlineStr">
         <is>
-          <t>analytics.fact_housing_observation|analytics.county_monthly_panel</t>
+          <t>analytics.fact_housing_observation|analytics.county_annual_controls</t>
         </is>
       </c>
       <c r="N5" s="3" t="inlineStr">
         <is>
-          <t>permits_5_plus_units</t>
+          <t>eviction_lab_filings_rate_estimate_annual|eviction_lab_households_threatened_rate_estimate_annual</t>
         </is>
       </c>
       <c r="O5" s="3" t="inlineStr">
         <is>
-          <t>proxy input</t>
+          <t>modeled annual</t>
         </is>
       </c>
       <c r="P5" s="3" t="inlineStr">
         <is>
-          <t>The sheet workaround is cumulative MF permits minus assumed completions over a rolling window; permit inputs are loaded, but the stock pipeline calculation is not implemented.</t>
+          <t>The official ETS Version 3.0 release was checked on 2026-08-16 and contains neither Los Angeles nor any California geography; the official observed/validated county analysis files also contain no LA County rows. The implementation therefore retains official Eviction Lab annual county modeled estimates for 2000-2018, with source-observation flags and 95% credible interval bounds preserved. No annual value is interpolated or expanded to monthly frequency, and the series is not direct local court filing data.</t>
         </is>
       </c>
       <c r="Q5" s="3" t="inlineStr"/>
@@ -986,18 +1010,18 @@
       <c r="X5" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="Y5" s="5" t="n">
-        <v>36556</v>
-      </c>
-      <c r="Z5" s="5" t="n">
-        <v>46173</v>
+      <c r="Y5" s="6" t="n">
+        <v>36891</v>
+      </c>
+      <c r="Z5" s="6" t="n">
+        <v>43465</v>
       </c>
       <c r="AA5" s="3" t="n">
-        <v>634</v>
+        <v>76</v>
       </c>
       <c r="AB5" s="3" t="inlineStr">
         <is>
-          <t>0 missing of 634 fact rows</t>
+          <t>0 missing of 76 fact rows</t>
         </is>
       </c>
       <c r="AC5" s="3" t="inlineStr">
@@ -1036,17 +1060,17 @@
           <t>Proxy using SFR permits in high-investor / rental-growth tracts or small MF permits.</t>
         </is>
       </c>
-      <c r="J6" s="3" t="inlineStr">
-        <is>
-          <t>Proxy input only</t>
-        </is>
-      </c>
-      <c r="K6" s="4" t="inlineStr">
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>Not implemented</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="inlineStr">
         <is>
           <t>census_bps_county|census_bps_state</t>
         </is>
       </c>
-      <c r="L6" s="4" t="inlineStr">
+      <c r="L6" s="5" t="inlineStr">
         <is>
           <t>permits_1_unit</t>
         </is>
@@ -1056,19 +1080,15 @@
           <t>analytics.fact_housing_observation|analytics.county_monthly_panel</t>
         </is>
       </c>
-      <c r="N6" s="3" t="inlineStr">
-        <is>
-          <t>permits_1_unit</t>
-        </is>
-      </c>
+      <c r="N6" s="3" t="inlineStr"/>
       <c r="O6" s="3" t="inlineStr">
         <is>
-          <t>proxy input</t>
+          <t>closed / not pursued</t>
         </is>
       </c>
       <c r="P6" s="3" t="inlineStr">
         <is>
-          <t>The sheet workaround needs SFR permits combined with investor/rental-growth tract logic; only 1-unit permits are loaded.</t>
+          <t>The approved decision keeps this target closed. Generic one-unit permits do not identify rental tenure or investor intent, and the repository does not invent an investor/rental-growth tract classifier. Reopen only if a qualifying official public source and explicit method are approved.</t>
         </is>
       </c>
       <c r="Q6" s="3" t="inlineStr"/>
@@ -1087,18 +1107,18 @@
       <c r="X6" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="Y6" s="5" t="n">
+      <c r="Y6" s="6" t="n">
         <v>36556</v>
       </c>
-      <c r="Z6" s="5" t="n">
-        <v>46173</v>
+      <c r="Z6" s="6" t="n">
+        <v>46203</v>
       </c>
       <c r="AA6" s="3" t="n">
-        <v>634</v>
+        <v>636</v>
       </c>
       <c r="AB6" s="3" t="inlineStr">
         <is>
-          <t>0 missing of 634 fact rows</t>
+          <t>0 missing of 636 fact rows</t>
         </is>
       </c>
       <c r="AC6" s="3" t="inlineStr">
@@ -1137,39 +1157,39 @@
           <t>Annual ACS change in occupied renter units; optionally interpolate or use CPS/HVS for state-level timing.</t>
         </is>
       </c>
-      <c r="J7" s="6" t="inlineStr">
+      <c r="J7" s="4" t="inlineStr">
         <is>
           <t>Partially implemented</t>
         </is>
       </c>
-      <c r="K7" s="4" t="inlineStr">
+      <c r="K7" s="5" t="inlineStr">
         <is>
           <t>census_acs_5year_b25003</t>
         </is>
       </c>
-      <c r="L7" s="4" t="inlineStr">
-        <is>
-          <t>acs_renter_occupied_units</t>
+      <c r="L7" s="5" t="inlineStr">
+        <is>
+          <t>net_change_occupied_apartments_annual|zcta_renter_occupied_units_vintage_change_annual</t>
         </is>
       </c>
       <c r="M7" s="3" t="inlineStr">
         <is>
-          <t>analytics.county_annual_controls|analytics.fact_housing_observation</t>
+          <t>analytics.county_annual_controls|analytics.zcta_annual_controls</t>
         </is>
       </c>
       <c r="N7" s="3" t="inlineStr">
         <is>
-          <t>acs_renter_occupied_units</t>
+          <t>net_change_occupied_apartments_annual</t>
         </is>
       </c>
       <c r="O7" s="3" t="inlineStr">
         <is>
-          <t>observed</t>
+          <t>proxy</t>
         </is>
       </c>
       <c r="P7" s="3" t="inlineStr">
         <is>
-          <t>ACS annual 5-year renter-occupied units are available; quarterly net change is not created.</t>
+          <t>Fourteen consecutive-vintage annual county differences are implemented for 2011-2024, and 3,562 exact-ZCTA differences are implemented for 2012-2024. Both are panel-only constructions from direct acs_renter_occupied_units inputs and are not fact observations. Adjacent ACS five-year estimates overlap for four survey years, so neither result is a one-year flow; no quarterly timing is created, and Census ZCTAs are not postal ZIPs.</t>
         </is>
       </c>
       <c r="Q7" s="3" t="inlineStr"/>
@@ -1180,26 +1200,26 @@
         <v>1</v>
       </c>
       <c r="V7" s="3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W7" s="3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X7" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="Y7" s="5" t="n">
+      <c r="Y7" s="6" t="n">
+        <v>40908</v>
+      </c>
+      <c r="Z7" s="6" t="n">
         <v>45657</v>
       </c>
-      <c r="Z7" s="5" t="n">
-        <v>45657</v>
-      </c>
       <c r="AA7" s="3" t="n">
-        <v>275</v>
+        <v>14</v>
       </c>
       <c r="AB7" s="3" t="inlineStr">
         <is>
-          <t>0 missing of 275 fact rows</t>
+          <t>0 missing of 14 panel cells</t>
         </is>
       </c>
       <c r="AC7" s="3" t="inlineStr">
@@ -1238,31 +1258,31 @@
           <t>Construct ratio using annual ACS income with interpolated or stepwise series.</t>
         </is>
       </c>
-      <c r="J8" s="6" t="inlineStr">
+      <c r="J8" s="4" t="inlineStr">
         <is>
           <t>Partially implemented</t>
         </is>
       </c>
-      <c r="K8" s="4" t="inlineStr">
+      <c r="K8" s="5" t="inlineStr">
         <is>
           <t>census_acs_5year_b19013|census_acs_5year_b25077</t>
         </is>
       </c>
-      <c r="L8" s="4" t="inlineStr">
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>county_annual_price_to_income_acs|zcta_annual_price_to_income_acs</t>
+        </is>
+      </c>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>analytics.county_annual_controls|analytics.zcta_annual_controls</t>
+        </is>
+      </c>
+      <c r="N8" s="3" t="inlineStr">
         <is>
           <t>county_annual_price_to_income_acs</t>
         </is>
       </c>
-      <c r="M8" s="3" t="inlineStr">
-        <is>
-          <t>analytics.county_annual_controls</t>
-        </is>
-      </c>
-      <c r="N8" s="3" t="inlineStr">
-        <is>
-          <t>county_annual_price_to_income_acs</t>
-        </is>
-      </c>
       <c r="O8" s="3" t="inlineStr">
         <is>
           <t>constructed</t>
@@ -1270,7 +1290,7 @@
       </c>
       <c r="P8" s="3" t="inlineStr">
         <is>
-          <t>Annual ACS ratio is implemented; quarterly/local alternatives are deferred.</t>
+          <t>Fifteen annual LA County ACS ratios are implemented for 2010-2024. Matched-vintage ratios are also implemented for the 274 configured Census ZCTAs for 2011-2024, with six source-null ZCTA-vintages preserved and 3,830 non-null ratios. Both ratios are panel-only constructions rather than fact observations. No quarterly timing is invented, and Census ZCTAs are not postal ZIPs.</t>
         </is>
       </c>
       <c r="Q8" s="3" t="inlineStr"/>
@@ -1281,7 +1301,7 @@
         <v>1</v>
       </c>
       <c r="V8" s="3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W8" s="3" t="b">
         <v>0</v>
@@ -1289,12 +1309,20 @@
       <c r="X8" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="Y8" s="3" t="inlineStr"/>
-      <c r="Z8" s="3" t="inlineStr"/>
+      <c r="Y8" s="6" t="n">
+        <v>40543</v>
+      </c>
+      <c r="Z8" s="6" t="n">
+        <v>45657</v>
+      </c>
       <c r="AA8" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB8" s="3" t="inlineStr"/>
+        <v>15</v>
+      </c>
+      <c r="AB8" s="3" t="inlineStr">
+        <is>
+          <t>0 missing of 15 panel cells</t>
+        </is>
+      </c>
       <c r="AC8" s="3" t="inlineStr">
         <is>
           <t>Review documented limitation before modeling</t>
@@ -1336,12 +1364,12 @@
           <t>Implemented with quarterly allocation</t>
         </is>
       </c>
-      <c r="K9" s="4" t="inlineStr">
+      <c r="K9" s="5" t="inlineStr">
         <is>
           <t>cdc_wonder_natality_county|cdc_wonder_ucd_1999_2020_la_county|cdc_wonder_ucd_2018_2024_county</t>
         </is>
       </c>
-      <c r="L9" s="4" t="inlineStr">
+      <c r="L9" s="5" t="inlineStr">
         <is>
           <t>cdc_wonder_live_births_annual|cdc_wonder_deaths_annual|natural_population_change_annual|natural_population_change_quarterly_allocated</t>
         </is>
@@ -1382,10 +1410,10 @@
       <c r="X9" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="Y9" s="5" t="n">
+      <c r="Y9" s="6" t="n">
         <v>39447</v>
       </c>
-      <c r="Z9" s="5" t="n">
+      <c r="Z9" s="6" t="n">
         <v>45657</v>
       </c>
       <c r="AA9" s="3" t="n">
@@ -1432,23 +1460,39 @@
           <t>Annual HUD PIT; no credible quarterly public alternative.</t>
         </is>
       </c>
-      <c r="J10" s="3" t="inlineStr">
-        <is>
-          <t>Not implemented</t>
-        </is>
-      </c>
-      <c r="K10" s="4" t="inlineStr"/>
-      <c r="L10" s="4" t="inlineStr"/>
-      <c r="M10" s="3" t="inlineStr"/>
-      <c r="N10" s="3" t="inlineStr"/>
+      <c r="J10" s="4" t="inlineStr">
+        <is>
+          <t>Partially implemented</t>
+        </is>
+      </c>
+      <c r="K10" s="5" t="inlineStr">
+        <is>
+          <t>hud_pit_coc_2007_2025</t>
+        </is>
+      </c>
+      <c r="L10" s="5" t="inlineStr">
+        <is>
+          <t>hud_pit_overall_homeless_annual|hud_pit_sheltered_homeless_annual|hud_pit_unsheltered_homeless_annual</t>
+        </is>
+      </c>
+      <c r="M10" s="3" t="inlineStr">
+        <is>
+          <t>analytics.fact_housing_observation|analytics.coc_annual_controls</t>
+        </is>
+      </c>
+      <c r="N10" s="3" t="inlineStr">
+        <is>
+          <t>hud_pit_overall_homeless_annual|hud_pit_sheltered_homeless_annual|hud_pit_unsheltered_homeless_annual</t>
+        </is>
+      </c>
       <c r="O10" s="3" t="inlineStr">
         <is>
-          <t>deferred</t>
+          <t>observed annual control</t>
         </is>
       </c>
       <c r="P10" s="3" t="inlineStr">
         <is>
-          <t>The sheet workaround specifies annual HUD PIT; HUD PIT/CoC data is not loaded.</t>
+          <t>The official HUD PIT annual 2007-2025 CoC source and explicit CA-600/606/607/612 project composite are implemented. The source is annual point-in-time only, the composite is not Los Angeles County, and row-level sheltered-only, partial-unsheltered, and no-count records remain analytically incomplete. Explicit geography-year rows remain in CoC annual controls even when all three analytical values are null; the requested high-frequency target is still unavailable.</t>
         </is>
       </c>
       <c r="Q10" s="3" t="inlineStr"/>
@@ -1456,23 +1500,31 @@
       <c r="S10" s="3" t="inlineStr"/>
       <c r="T10" s="3" t="inlineStr"/>
       <c r="U10" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V10" s="3" t="b">
         <v>0</v>
       </c>
       <c r="W10" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X10" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="Y10" s="3" t="inlineStr"/>
-      <c r="Z10" s="3" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="Y10" s="6" t="n">
+        <v>39447</v>
+      </c>
+      <c r="Z10" s="6" t="n">
+        <v>46022</v>
+      </c>
       <c r="AA10" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB10" s="3" t="inlineStr"/>
+        <v>22350</v>
+      </c>
+      <c r="AB10" s="3" t="inlineStr">
+        <is>
+          <t>1742 missing of 22350 fact rows</t>
+        </is>
+      </c>
       <c r="AC10" s="3" t="inlineStr">
         <is>
           <t>Review documented limitation before modeling</t>
@@ -1517,39 +1569,23 @@
       </c>
       <c r="H11" s="3" t="inlineStr"/>
       <c r="I11" s="3" t="inlineStr"/>
-      <c r="J11" s="6" t="inlineStr">
-        <is>
-          <t>Partially implemented – ACS annual availability and HUD/USPS quarterly proxies; monthly listings unavailable</t>
-        </is>
-      </c>
-      <c r="K11" s="4" t="inlineStr">
-        <is>
-          <t>census_acs_5year_b25003|census_acs_5year_b25004|hud_usps_ncwm_quarterly</t>
-        </is>
-      </c>
-      <c r="L11" s="4" t="inlineStr">
-        <is>
-          <t>acs_renter_occupied_units|acs_renter_occupied_units_moe|acs_for_rent_vacant_units|acs_for_rent_vacant_units_moe|acs_rental_availability_rate|usps_total_residential_addresses|usps_short_term_vacant_residential_addresses|usps_long_term_vacant_residential_addresses|usps_vacant_residential_addresses|usps_no_stat_residential_addresses|usps_active_residential_addresses|usps_residential_vacancy_rate|usps_residential_no_stat_rate</t>
-        </is>
-      </c>
-      <c r="M11" s="3" t="inlineStr">
-        <is>
-          <t>analytics.fact_housing_observation|analytics.county_annual_controls|data/restricted/hud_usps/active/ca_county_quarterly.parquet|data/restricted/hud_usps/active/la_tract_2020_quarterly.parquet|data/restricted/hud_usps/active/la_postal_zip_county_part_quarterly.parquet|data/restricted/hud_usps/active/long_observations_with_lineage.parquet</t>
-        </is>
-      </c>
-      <c r="N11" s="3" t="inlineStr">
-        <is>
-          <t>acs_renter_occupied_units|acs_renter_occupied_units_moe|acs_for_rent_vacant_units|acs_for_rent_vacant_units_moe|acs_rental_availability_rate|usps_total_residential_addresses|usps_short_term_vacant_residential_addresses|usps_long_term_vacant_residential_addresses|usps_vacant_residential_addresses|usps_no_stat_residential_addresses|usps_active_residential_addresses|usps_residential_vacancy_rate|usps_residential_no_stat_rate</t>
-        </is>
-      </c>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>Not implemented</t>
+        </is>
+      </c>
+      <c r="K11" s="5" t="inlineStr"/>
+      <c r="L11" s="5" t="inlineStr"/>
+      <c r="M11" s="3" t="inlineStr"/>
+      <c r="N11" s="3" t="inlineStr"/>
       <c r="O11" s="3" t="inlineStr">
         <is>
-          <t>separate annual and quarterly proxies</t>
+          <t>unavailable target</t>
         </is>
       </c>
       <c r="P11" s="3" t="inlineStr">
         <is>
-          <t>The annual ACS rental-availability proxy is for-rent vacant units divided by renter-occupied plus for-rent vacant units, using matched B25003 and B25004 estimates. Component 90% margins of error are retained, and unreliable county ratios are suppressed. Direct ACS counts and margins of error are retained at county and ZCTA geography; ZCTAs are not postal ZIPs. The eight active HUD-USPS variables are native-quarterly only and remain a separate all-residential measure. The vacancy proxy is (short-term vacant + long-term vacant) / total residential addresses, while no-stat remains a separate diagnostic. Direct provider components are observed at standardized 2020-tract geography; California county aggregates are constructed, and Los Angeles County postal-ZIP county-parts are modeled with the fixed 2026 Q1 crosswalk. Detailed tract and modeled ZIP-part derivatives remain access-controlled under the HUD-USPS sublicense. This is not true rental-listing inventory; ZORI is not inventory (it is a rent index), and Redfin for-sale active listings are not a valid substitute. The monthly rental-listing series remains missing at documented source and license acquisition. The former derived package file was deleted; its historical quarantine manifest is superseded and is not an active input.</t>
+          <t>The annual ACS rental-availability proxy is for-rent vacant units divided by renter-occupied plus for-rent vacant units, using matched B25003 and B25004 estimates. Component 90% margins of error are retained, and unreliable county ratios are suppressed. Direct ACS counts and margins of error are retained at county and ZCTA geography; ZCTAs are not postal ZIPs. The eight active HUD-USPS variables are native-quarterly only and remain a separate all-residential measure. The vacancy proxy is (short-term vacant + long-term vacant) / total residential addresses, while no-stat remains a separate diagnostic. Direct provider components are observed at standardized 2020-tract geography; California county aggregates are constructed, and Los Angeles County postal-ZIP county-parts are modeled with the fixed 2026 Q1 crosswalk. Detailed tract and modeled ZIP-part derivatives remain access-controlled under the HUD-USPS sublicense. This is not true rental-listing inventory; ZORI is not inventory (it is a rent index), and Redfin for-sale active listings are not a valid substitute. The governing methodology names no approved source for the true monthly rental-listing series, so the blocker is a methodology/source-identification decision rather than a credential or coding step. The former derived package file was deleted; its historical quarantine manifest is superseded and is not an active input.</t>
         </is>
       </c>
       <c r="Q11" s="3" t="inlineStr"/>
@@ -1557,342 +1593,31 @@
       <c r="S11" s="3" t="inlineStr"/>
       <c r="T11" s="3" t="inlineStr"/>
       <c r="U11" s="3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V11" s="3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W11" s="3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X11" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y11" s="5" t="n">
-        <v>39538</v>
-      </c>
-      <c r="Z11" s="5" t="n">
-        <v>46112</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Y11" s="3" t="inlineStr"/>
+      <c r="Z11" s="3" t="inlineStr"/>
       <c r="AA11" s="3" t="n">
-        <v>1770036</v>
-      </c>
-      <c r="AB11" s="3" t="inlineStr">
-        <is>
-          <t>9256 missing of 1770036 fact rows</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AB11" s="3" t="inlineStr"/>
       <c r="AC11" s="3" t="inlineStr">
-        <is>
-          <t>Review documented limitation before modeling</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>AVAILABLE VARIABLES - Overall Housing Market</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>Price-to-Rent Ratio</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>Price-to-Rent Ratio</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>Constructed from FHFA / ZORI</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>Monthly / Quarterly</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr"/>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t>Very clean once inputs chosen</t>
-        </is>
-      </c>
-      <c r="H12" s="3" t="inlineStr"/>
-      <c r="I12" s="3" t="inlineStr"/>
-      <c r="J12" s="3" t="inlineStr">
-        <is>
-          <t>Partially implemented - alternate source</t>
-        </is>
-      </c>
-      <c r="K12" s="4" t="inlineStr">
-        <is>
-          <t>zillow_county_zhvi|zillow_county_zori_smoothed_sa</t>
-        </is>
-      </c>
-      <c r="L12" s="4" t="inlineStr">
-        <is>
-          <t>price_to_rent_ratio</t>
-        </is>
-      </c>
-      <c r="M12" s="3" t="inlineStr">
-        <is>
-          <t>analytics.county_monthly_panel</t>
-        </is>
-      </c>
-      <c r="N12" s="3" t="inlineStr">
-        <is>
-          <t>price_to_rent_ratio</t>
-        </is>
-      </c>
-      <c r="O12" s="3" t="inlineStr">
-        <is>
-          <t>constructed</t>
-        </is>
-      </c>
-      <c r="P12" s="3" t="inlineStr">
-        <is>
-          <t>The active monthly panel ratio uses ZHVI/ZORI. The sheet specifies FHFA/ZORI; that version needs an explicit FHFA index-to-rent construction choice and is not yet implemented.</t>
-        </is>
-      </c>
-      <c r="Q12" s="3" t="inlineStr"/>
-      <c r="R12" s="3" t="inlineStr"/>
-      <c r="S12" s="3" t="inlineStr"/>
-      <c r="T12" s="3" t="inlineStr"/>
-      <c r="U12" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="V12" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="W12" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="X12" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y12" s="3" t="inlineStr"/>
-      <c r="Z12" s="3" t="inlineStr"/>
-      <c r="AA12" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB12" s="3" t="inlineStr"/>
-      <c r="AC12" s="3" t="inlineStr">
-        <is>
-          <t>Review documented limitation before modeling</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>AVAILABLE VARIABLES - Overall Housing Market</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>Housing Turnover</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>Housing Turnover</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>Redfin (sales / inventory)</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>Monthly</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr"/>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>Useful liquidity metric</t>
-        </is>
-      </c>
-      <c r="H13" s="3" t="inlineStr"/>
-      <c r="I13" s="3" t="inlineStr"/>
-      <c r="J13" s="6" t="inlineStr">
-        <is>
-          <t>Partially implemented</t>
-        </is>
-      </c>
-      <c r="K13" s="4" t="inlineStr">
-        <is>
-          <t>redfin_county_monthly</t>
-        </is>
-      </c>
-      <c r="L13" s="4" t="inlineStr">
-        <is>
-          <t>sales_to_inventory_ratio|inventory_to_sales_ratio</t>
-        </is>
-      </c>
-      <c r="M13" s="3" t="inlineStr">
-        <is>
-          <t>analytics.county_monthly_panel</t>
-        </is>
-      </c>
-      <c r="N13" s="3" t="inlineStr">
-        <is>
-          <t>sales_to_inventory_ratio|inventory_to_sales_ratio</t>
-        </is>
-      </c>
-      <c r="O13" s="3" t="inlineStr">
-        <is>
-          <t>constructed</t>
-        </is>
-      </c>
-      <c r="P13" s="3" t="inlineStr">
-        <is>
-          <t>Sales/inventory liquidity is implemented; sales/housing-stock turnover is deferred.</t>
-        </is>
-      </c>
-      <c r="Q13" s="3" t="inlineStr"/>
-      <c r="R13" s="3" t="inlineStr"/>
-      <c r="S13" s="3" t="inlineStr"/>
-      <c r="T13" s="3" t="inlineStr"/>
-      <c r="U13" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="V13" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="W13" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="X13" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y13" s="3" t="inlineStr"/>
-      <c r="Z13" s="3" t="inlineStr"/>
-      <c r="AA13" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB13" s="3" t="inlineStr"/>
-      <c r="AC13" s="3" t="inlineStr">
-        <is>
-          <t>Review documented limitation before modeling</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>Population, Labor, Macro Controls</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>Personal Income (proxy)</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>Personal Income (proxy)</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>BEA</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr">
-        <is>
-          <t>Quarterly</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>county quarterly limited</t>
-        </is>
-      </c>
-      <c r="G14" s="3" t="inlineStr">
-        <is>
-          <t>State is clean; county is noisier</t>
-        </is>
-      </c>
-      <c r="H14" s="3" t="inlineStr"/>
-      <c r="I14" s="3" t="inlineStr"/>
-      <c r="J14" s="6" t="inlineStr">
-        <is>
-          <t>Partially implemented</t>
-        </is>
-      </c>
-      <c r="K14" s="4" t="inlineStr">
-        <is>
-          <t>bea_state_personal_income|bea_county_personal_income</t>
-        </is>
-      </c>
-      <c r="L14" s="4" t="inlineStr">
-        <is>
-          <t>bea_ca_personal_income_q_sa|bea_la_county_personal_income_annual</t>
-        </is>
-      </c>
-      <c r="M14" s="3" t="inlineStr">
-        <is>
-          <t>analytics.state_quarterly_panel|analytics.county_annual_controls</t>
-        </is>
-      </c>
-      <c r="N14" s="3" t="inlineStr">
-        <is>
-          <t>bea_ca_personal_income_q_sa|bea_la_county_personal_income_annual</t>
-        </is>
-      </c>
-      <c r="O14" s="3" t="inlineStr">
-        <is>
-          <t>observed</t>
-        </is>
-      </c>
-      <c r="P14" s="3" t="inlineStr">
-        <is>
-          <t>Aligned with BEA as the sheet source. State quarterly is loaded; county is annual because county quarterly personal income is limited/noisier as noted in the sheet.</t>
-        </is>
-      </c>
-      <c r="Q14" s="3" t="inlineStr"/>
-      <c r="R14" s="3" t="inlineStr"/>
-      <c r="S14" s="3" t="inlineStr"/>
-      <c r="T14" s="3" t="inlineStr"/>
-      <c r="U14" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="V14" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="W14" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="X14" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y14" s="5" t="n">
-        <v>17623</v>
-      </c>
-      <c r="Z14" s="5" t="n">
-        <v>46112</v>
-      </c>
-      <c r="AA14" s="3" t="n">
-        <v>369</v>
-      </c>
-      <c r="AB14" s="3" t="inlineStr">
-        <is>
-          <t>0 missing of 369 fact rows</t>
-        </is>
-      </c>
-      <c r="AC14" s="3" t="inlineStr">
         <is>
           <t>Review documented limitation before modeling</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AC14"/>
+  <autoFilter ref="A1:AC11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>